<commit_message>
Pipeline run results - 2026-04-30 16:50:41 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-1012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777567820.png</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>The jeans display multiple large intentional-style rips and tears throughout both legs, along with white paint-like staining and distressed fabric damage across the entire garment.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove generate_images from pipeline, cache pip, faster polling
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,71 +1222,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ORD-1012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sean Kelly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Jeans</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>submissions/jeans_1777567820.png</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>ELIGIBLE FOR AI INSPECTION</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>tear</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>The jeans display multiple large intentional-style rips and tears throughout both legs, along with white paint-like staining and distressed fabric damage across the entire garment.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 17:22:41 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-1012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777569741.png</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>The jeans display multiple large intentional-looking rips, holes, and frayed tears across both legs, along with what appears to be paint-like staining, making this item unsuitable for approval regardless of potential designer distressing intent.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Increase polling wait to 60s initial, 6min total timeout
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,71 +1222,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ORD-1012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sean Kelly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Jeans</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>submissions/jeans_1777569741.png</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>ELIGIBLE FOR AI INSPECTION</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>tear</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>The jeans display multiple large intentional-looking rips, holes, and frayed tears across both legs, along with what appears to be paint-like staining, making this item unsuitable for approval regardless of potential designer distressing intent.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 17:34:52 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-1012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777570469.png</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>The jeans exhibit multiple large intentional-style rips, tears, and heavily distressed areas across both legs, along with what appears to be paint staining on the fabric surface.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix polling: filter by pipeline.yml only, fix timeout message
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,71 +1222,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ORD-1012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sean Kelly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Jeans</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>submissions/jeans_1777570469.png</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>ELIGIBLE FOR AI INSPECTION</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>tear</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>The jeans exhibit multiple large intentional-style rips, tears, and heavily distressed areas across both legs, along with what appears to be paint staining on the fabric surface.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 17:54:17 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-1012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777571635.png</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>The jeans exhibit multiple large intentional-style rips and tears across both legs, along with visible paint-like staining/discolouration throughout the fabric.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix REPO detection: hardcode owner/repo instead of URL parsing
getRepoInfo() only worked on github.io URLs. On Vercel the hostname
is different so REPO was empty, silently breaking all API calls.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,71 +1222,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ORD-1012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Sean Kelly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Jeans</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>submissions/jeans_1777571635.png</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>ELIGIBLE FOR AI INSPECTION</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>REJECT</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>tear</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>The jeans exhibit multiple large intentional-style rips and tears across both legs, along with visible paint-like staining/discolouration throughout the fabric.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 18:11:07 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Returns_Queue" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,71 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-1012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777572644.png</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>The jeans display multiple large intentional-style rips, holes, and frayed tears across both legs, along with visible paint-like staining/discolouration throughout the fabric.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 22:45:47 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1287,6 +1287,71 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORD-1013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sean Kelly</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777589130.png</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>The jeans display multiple large intentional-style rips, holes, and frayed tears throughout the legs, along with what appears to be paint-like staining/discolouration across the fabric.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-04-30 23:21:47 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1352,6 +1352,71 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ORD-1014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777591290.png</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>The jeans exhibit multiple large intentional-style rips, holes, and frayed fabric tears across both legs, along with visible paint-like staining/discolouration throughout the fabric.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pipeline run results - 2026-05-01 00:00:55 UTC
</commit_message>
<xml_diff>
--- a/data/Returns_Queue.xlsx
+++ b/data/Returns_Queue.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1417,6 +1417,71 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ORD-1015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SALLEY KELLY</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Jeans</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>submissions/jeans_1777593634.png</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>ELIGIBLE FOR AI INSPECTION</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>REJECT</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>tear</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>The jeans display multiple large intentional-style rips and tears across both legs, along with paint-like splatter marks and heavily distressed fabric throughout the garment.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>